<commit_message>
V7.2: cifras superadas retiradas de cifras_clave (una sola cifra de déficit con bajas), construcción adicional con dosis no nula, f2 no difundible, comparadores de R5 rotulados, GSADF nacional reverificado y ficha de burbuja
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GDwCFFTud391ebBMaJpdsw
</commit_message>
<xml_diff>
--- a/output/v7/tablas_regionales.xlsx
+++ b/output/v7/tablas_regionales.xlsx
@@ -1873,7 +1873,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -2905,7 +2905,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -3416,7 +3416,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -3917,7 +3917,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -4438,7 +4438,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4939,7 +4939,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -4949,7 +4949,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -5450,7 +5450,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5460,7 +5460,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -5961,7 +5961,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5971,7 +5971,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -6472,7 +6472,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -6482,7 +6482,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -6993,7 +6993,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -8005,7 +8005,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -8015,7 +8015,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -8516,7 +8516,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -8526,7 +8526,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -9037,7 +9037,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -9538,7 +9538,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -9548,7 +9548,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -10049,7 +10049,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RMSE base exigente ×100</t>
+          <t>RMSE base más exigente ×100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -10059,7 +10059,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>¿Bate?</t>
+          <t>¿Bate a la base más exigente?</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">

</xml_diff>